<commit_message>
Shorts phase 1 (work in progress): the short reads the workbook
The short's cards fill from the operator's workbook: one metric a card,
the implied-growth card, the 52-week and short-interest cards, the quarter
cards and the print against consensus, the release opened from the News
sheet link and the wires, a company picture, the clear area, and Dennis in
the macro short. Not for merge until the re-rendered frames are approved.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PtFQaojNjukBZRpdj68CaY
</commit_message>
<xml_diff>
--- a/fixtures/company_data/dennis_data.xlsx
+++ b/fixtures/company_data/dennis_data.xlsx
@@ -2466,7 +2466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3273,6 +3273,129 @@
         <v>-0.066</v>
       </c>
       <c r="K22" t="inlineStr">
+        <is>
+          <t>computed</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>eps_street</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>EPS actual (street basis)</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>computed</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>eps_consensus</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>EPS estimate (mean)</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>computed</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>revenue_consensus</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Revenue estimate (mean)</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>110000000</v>
+      </c>
+      <c r="D25" t="n">
+        <v>117000000</v>
+      </c>
+      <c r="E25" t="n">
+        <v>122000000</v>
+      </c>
+      <c r="F25" t="n">
+        <v>137000000</v>
+      </c>
+      <c r="G25" t="n">
+        <v>115000000</v>
+      </c>
+      <c r="H25" t="n">
+        <v>118000000</v>
+      </c>
+      <c r="I25" t="n">
+        <v>121000000</v>
+      </c>
+      <c r="J25" t="n">
+        <v>138000000</v>
+      </c>
+      <c r="K25" t="inlineStr">
         <is>
           <t>computed</t>
         </is>
@@ -4719,7 +4842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4856,6 +4979,26 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Example Corp announces AI partnership with a cloud provider</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Business Wire</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://example.com/news/ai-partnership</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>